<commit_message>
Fixed demo code and output
</commit_message>
<xml_diff>
--- a/outputs/VIT_output.xlsx
+++ b/outputs/VIT_output.xlsx
@@ -1024,7 +1024,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>healthy</t>
+          <t>cordona</t>
         </is>
       </c>
     </row>
@@ -1036,7 +1036,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>healthy</t>
+          <t>cordona</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>healthy</t>
+          <t>cordona</t>
         </is>
       </c>
     </row>
@@ -1060,7 +1060,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>healthy</t>
+          <t>cordona</t>
         </is>
       </c>
     </row>
@@ -1072,7 +1072,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>healthy</t>
+          <t>cordona</t>
         </is>
       </c>
     </row>
@@ -1084,7 +1084,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>healthy</t>
+          <t>cordona</t>
         </is>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>healthy</t>
+          <t>cordona</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1108,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>healthy</t>
+          <t>cordona</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>healthy</t>
+          <t>cordona</t>
         </is>
       </c>
     </row>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>healthy</t>
+          <t>cordona</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1144,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>healthy</t>
+          <t>cordona</t>
         </is>
       </c>
     </row>
@@ -1156,7 +1156,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>healthy</t>
+          <t>cordona</t>
         </is>
       </c>
     </row>
@@ -1168,7 +1168,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>healthy</t>
+          <t>cordona</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>healthy</t>
+          <t>cordona</t>
         </is>
       </c>
     </row>
@@ -1192,7 +1192,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>healthy</t>
+          <t>cordona</t>
         </is>
       </c>
     </row>
@@ -1204,7 +1204,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>healthy</t>
+          <t>cordona</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>cordona</t>
+          <t>healthy</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>cordona</t>
+          <t>healthy</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1240,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>cordona</t>
+          <t>healthy</t>
         </is>
       </c>
     </row>
@@ -1252,7 +1252,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>cordona</t>
+          <t>healthy</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>cordona</t>
+          <t>healthy</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>cordona</t>
+          <t>healthy</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>cordona</t>
+          <t>healthy</t>
         </is>
       </c>
     </row>
@@ -1312,7 +1312,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>cordona</t>
+          <t>healthy</t>
         </is>
       </c>
     </row>
@@ -1324,7 +1324,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>cordona</t>
+          <t>healthy</t>
         </is>
       </c>
     </row>
@@ -1336,7 +1336,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>cordona</t>
+          <t>healthy</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>cordona</t>
+          <t>healthy</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>cordona</t>
+          <t>healthy</t>
         </is>
       </c>
     </row>

</xml_diff>